<commit_message>
Parse weekly grid timetables (Time x weekday columns).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Client/public/sample-centre-timetable.xlsx
+++ b/Client/public/sample-centre-timetable.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timetable" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Timetable" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,384 +417,376 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Subject</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Month</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Saturday</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>09:30–10:15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>09:00 - 10:30</t>
+          <t>Chemistry</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>English Language</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Legal Reasoning</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>10:15–11:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>11:00 - 12:30</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>July 2026</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Quantitative Aptitude</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Logical Reasoning</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>11:15–12:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>Chemistry</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>14:00 - 15:30</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>July 2026</t>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Reasoning Ability</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>English Language</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>12:00–12:45</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>Physics Revision</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>09:00 - 10:30</t>
+          <t>Numericals</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Formula Revision</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>General Awareness</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Current Affairs &amp; GK</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>01:30–02:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>11:00 - 12:30</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Lunch</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>02:15–03:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>Mathematics Practice</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>09:00 - 10:30</t>
+          <t>Chemistry Practice</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Problem Solving</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>Biology Practice</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Computer Knowledge</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Quantitative Techniques</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>03:15–04:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>Doubt Session</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11:00 - 12:30</t>
+          <t>Test Discussion</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Mock Test</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>Reasoning Skills</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Mock Test</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>04:00–04:45</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>Mock Quiz</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14:00 - 15:30</t>
+          <t>PYQs</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>July 2026</t>
+          <t>Current Affairs</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Career Guidance</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>04:45–05:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>Self Study</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>09:00 - 10:30</t>
+          <t>Self Study</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>Self Study</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>11:00 - 12:30</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Chemistry</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>09:00 - 10:30</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>11:00 - 12:30</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>July 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>14:00 - 15:30</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>July 2026</t>
+          <t>Self Study</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Self Study</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Weekly Revision</t>
         </is>
       </c>
     </row>

</xml_diff>